<commit_message>
WIP: valida caja contra Excel y evita cobros al cambiar de modelo
</commit_message>
<xml_diff>
--- a/tests/oracle/ORACULO_sim2.xlsx
+++ b/tests/oracle/ORACULO_sim2.xlsx
@@ -4444,7 +4444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EZ7"/>
+  <dimension ref="A1:GV7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="184" min="1" max="1"/>
@@ -5386,6 +5386,246 @@
           <t>CONS-08</t>
         </is>
       </c>
+      <c r="FA1" t="inlineStr">
+        <is>
+          <t>capitalInicial</t>
+        </is>
+      </c>
+      <c r="FB1" t="inlineStr">
+        <is>
+          <t>compraActivos</t>
+        </is>
+      </c>
+      <c r="FC1" t="inlineStr">
+        <is>
+          <t>adquisicionNeta</t>
+        </is>
+      </c>
+      <c r="FD1" t="inlineStr">
+        <is>
+          <t>valorCompradoNeto</t>
+        </is>
+      </c>
+      <c r="FE1" t="inlineStr">
+        <is>
+          <t>valorInventarioNeto</t>
+        </is>
+      </c>
+      <c r="FF1" t="inlineStr">
+        <is>
+          <t>cajaInicial</t>
+        </is>
+      </c>
+      <c r="FG1" t="inlineStr">
+        <is>
+          <t>tasaNuevoPrestamo</t>
+        </is>
+      </c>
+      <c r="FH1" t="inlineStr">
+        <is>
+          <t>interesMensual</t>
+        </is>
+      </c>
+      <c r="FI1" t="inlineStr">
+        <is>
+          <t>tasaMensual</t>
+        </is>
+      </c>
+      <c r="FJ1" t="inlineStr">
+        <is>
+          <t>intereses</t>
+        </is>
+      </c>
+      <c r="FK1" t="inlineStr">
+        <is>
+          <t>pagosOperacion</t>
+        </is>
+      </c>
+      <c r="FL1" t="inlineStr">
+        <is>
+          <t>cajaFinal</t>
+        </is>
+      </c>
+      <c r="FM1" t="inlineStr">
+        <is>
+          <t>depreciacionAcumulada</t>
+        </is>
+      </c>
+      <c r="FN1" t="inlineStr">
+        <is>
+          <t>activosCosto</t>
+        </is>
+      </c>
+      <c r="FO1" t="inlineStr">
+        <is>
+          <t>activosFijos</t>
+        </is>
+      </c>
+      <c r="FP1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.ingresos</t>
+        </is>
+      </c>
+      <c r="FQ1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.ventasNetas</t>
+        </is>
+      </c>
+      <c r="FR1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.costos</t>
+        </is>
+      </c>
+      <c r="FS1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.utilidad</t>
+        </is>
+      </c>
+      <c r="FT1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.depreciacion</t>
+        </is>
+      </c>
+      <c r="FU1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.intereses</t>
+        </is>
+      </c>
+      <c r="FV1" t="inlineStr">
+        <is>
+          <t>financial.estadoResultados.costosProduccion</t>
+        </is>
+      </c>
+      <c r="FW1" t="inlineStr">
+        <is>
+          <t>financial.balanceCaja.cajaInicial</t>
+        </is>
+      </c>
+      <c r="FX1" t="inlineStr">
+        <is>
+          <t>financial.balanceCaja.entradas</t>
+        </is>
+      </c>
+      <c r="FY1" t="inlineStr">
+        <is>
+          <t>financial.balanceCaja.salidas</t>
+        </is>
+      </c>
+      <c r="FZ1" t="inlineStr">
+        <is>
+          <t>financial.balanceCaja.cajaFinal</t>
+        </is>
+      </c>
+      <c r="GA1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.cajaInicial</t>
+        </is>
+      </c>
+      <c r="GB1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.cobrosVentas</t>
+        </is>
+      </c>
+      <c r="GC1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.pagosOperacion</t>
+        </is>
+      </c>
+      <c r="GD1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.compraActivos</t>
+        </is>
+      </c>
+      <c r="GE1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.financiamiento</t>
+        </is>
+      </c>
+      <c r="GF1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.operacion</t>
+        </is>
+      </c>
+      <c r="GG1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.inversion</t>
+        </is>
+      </c>
+      <c r="GH1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.flujoNeto</t>
+        </is>
+      </c>
+      <c r="GI1" t="inlineStr">
+        <is>
+          <t>financial.flujoCaja.cajaFinal</t>
+        </is>
+      </c>
+      <c r="GJ1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.efectivo</t>
+        </is>
+      </c>
+      <c r="GK1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.activosFijos</t>
+        </is>
+      </c>
+      <c r="GL1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.inventarioMP</t>
+        </is>
+      </c>
+      <c r="GM1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.activos</t>
+        </is>
+      </c>
+      <c r="GN1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.deuda</t>
+        </is>
+      </c>
+      <c r="GO1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.patrimonio</t>
+        </is>
+      </c>
+      <c r="GP1" t="inlineStr">
+        <is>
+          <t>financial.balanceGeneral.pasivoPatrimonio</t>
+        </is>
+      </c>
+      <c r="GQ1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.montoPrestamo</t>
+        </is>
+      </c>
+      <c r="GR1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.tasaTEA</t>
+        </is>
+      </c>
+      <c r="GS1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.deudaPrincipal</t>
+        </is>
+      </c>
+      <c r="GT1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.tasaAdicionalProximoPrestamo</t>
+        </is>
+      </c>
+      <c r="GU1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.tasaMensual</t>
+        </is>
+      </c>
+      <c r="GV1" t="inlineStr">
+        <is>
+          <t>financial.financiamiento.intereses</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -5976,6 +6216,197 @@
       </c>
       <c r="EZ2" s="0">
         <f>AND(K2=0,AF2&lt;5)</f>
+        <v/>
+      </c>
+      <c r="FA2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB2">
+        <f>1*2500*(1+0.03+0.02)+1*3500*(1+0.03+0.02)+1*1200*(1+0.03+0.02)+1*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC2">
+        <f>1*2500+1*3500+1*1200+1*300</f>
+        <v/>
+      </c>
+      <c r="FD2">
+        <f>(CF2*25+CH2*45+CJ2*80+CL2*4+CN2*9+CP2*2+CR2*4+CT2*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FE2">
+        <f>(DC2*25+DE2*45+DG2*80+DJ2*4+DL2*9+DO2*2+DQ2*4+DS2*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FF2">
+        <f>FA2</f>
+        <v/>
+      </c>
+      <c r="FG2">
+        <f>(1+AR2/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH2">
+        <f>0*0+AP2*FG2</f>
+        <v/>
+      </c>
+      <c r="FI2">
+        <f>IFERROR(FH2/(0+AP2),0)</f>
+        <v/>
+      </c>
+      <c r="FJ2">
+        <f>FH2*1</f>
+        <v/>
+      </c>
+      <c r="FK2">
+        <f>EQ2-DW2-DU2+FD2+FJ2</f>
+        <v/>
+      </c>
+      <c r="FL2">
+        <f>FF2+EK2+AP2-FK2-FB2</f>
+        <v/>
+      </c>
+      <c r="FM2">
+        <f>0+DW2</f>
+        <v/>
+      </c>
+      <c r="FN2">
+        <f>0+FC2</f>
+        <v/>
+      </c>
+      <c r="FO2">
+        <f>FN2-FM2</f>
+        <v/>
+      </c>
+      <c r="FP2">
+        <f>EK2</f>
+        <v/>
+      </c>
+      <c r="FQ2">
+        <f>EK2</f>
+        <v/>
+      </c>
+      <c r="FR2">
+        <f>EQ2+FJ2</f>
+        <v/>
+      </c>
+      <c r="FS2">
+        <f>ER2-FJ2</f>
+        <v/>
+      </c>
+      <c r="FT2">
+        <f>DW2</f>
+        <v/>
+      </c>
+      <c r="FU2">
+        <f>FJ2</f>
+        <v/>
+      </c>
+      <c r="FV2">
+        <f>EQ2</f>
+        <v/>
+      </c>
+      <c r="FW2">
+        <f>FF2</f>
+        <v/>
+      </c>
+      <c r="FX2">
+        <f>EK2+AP2</f>
+        <v/>
+      </c>
+      <c r="FY2">
+        <f>FK2+FB2</f>
+        <v/>
+      </c>
+      <c r="FZ2">
+        <f>FL2</f>
+        <v/>
+      </c>
+      <c r="GA2">
+        <f>FF2</f>
+        <v/>
+      </c>
+      <c r="GB2">
+        <f>EK2</f>
+        <v/>
+      </c>
+      <c r="GC2">
+        <f>FK2</f>
+        <v/>
+      </c>
+      <c r="GD2">
+        <f>FB2</f>
+        <v/>
+      </c>
+      <c r="GE2">
+        <f>AP2</f>
+        <v/>
+      </c>
+      <c r="GF2">
+        <f>EK2-FK2</f>
+        <v/>
+      </c>
+      <c r="GG2">
+        <f>-FB2</f>
+        <v/>
+      </c>
+      <c r="GH2">
+        <f>FL2-FF2</f>
+        <v/>
+      </c>
+      <c r="GI2">
+        <f>FL2</f>
+        <v/>
+      </c>
+      <c r="GJ2">
+        <f>FL2</f>
+        <v/>
+      </c>
+      <c r="GK2">
+        <f>FO2</f>
+        <v/>
+      </c>
+      <c r="GL2">
+        <f>FE2</f>
+        <v/>
+      </c>
+      <c r="GM2">
+        <f>FL2+FO2+FE2</f>
+        <v/>
+      </c>
+      <c r="GN2">
+        <f>AS2</f>
+        <v/>
+      </c>
+      <c r="GO2">
+        <f>FL2+FO2+FE2-AS2</f>
+        <v/>
+      </c>
+      <c r="GP2">
+        <f>FL2+FO2+FE2</f>
+        <v/>
+      </c>
+      <c r="GQ2">
+        <f>AP2</f>
+        <v/>
+      </c>
+      <c r="GR2">
+        <f>AR2</f>
+        <v/>
+      </c>
+      <c r="GS2">
+        <f>AS2</f>
+        <v/>
+      </c>
+      <c r="GT2">
+        <f>AT2</f>
+        <v/>
+      </c>
+      <c r="GU2">
+        <f>FI2</f>
+        <v/>
+      </c>
+      <c r="GV2">
+        <f>FJ2</f>
         <v/>
       </c>
     </row>
@@ -6554,6 +6985,197 @@
         <f>AND(K3=0,AF3&lt;5)</f>
         <v/>
       </c>
+      <c r="FA3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB3">
+        <f>1*2500*(1+0.03+0.02)+1*3500*(1+0.03+0.02)+1*1200*(1+0.03+0.02)+1*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC3">
+        <f>1*2500+1*3500+1*1200+1*300</f>
+        <v/>
+      </c>
+      <c r="FD3">
+        <f>(CF3*25+CH3*45+CJ3*80+CL3*4+CN3*9+CP3*2+CR3*4+CT3*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FE3">
+        <f>(DC3*25+DE3*45+DG3*80+DJ3*4+DL3*9+DO3*2+DQ3*4+DS3*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF3">
+        <f>FA3</f>
+        <v/>
+      </c>
+      <c r="FG3">
+        <f>(1+AR3/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH3">
+        <f>0*0+AP3*FG3</f>
+        <v/>
+      </c>
+      <c r="FI3">
+        <f>IFERROR(FH3/(0+AP3),0)</f>
+        <v/>
+      </c>
+      <c r="FJ3">
+        <f>FH3*1</f>
+        <v/>
+      </c>
+      <c r="FK3">
+        <f>EQ3-DW3-DU3+FD3+FJ3</f>
+        <v/>
+      </c>
+      <c r="FL3">
+        <f>FF3+EK3+AP3-FK3-FB3</f>
+        <v/>
+      </c>
+      <c r="FM3">
+        <f>0+DW3</f>
+        <v/>
+      </c>
+      <c r="FN3">
+        <f>0+FC3</f>
+        <v/>
+      </c>
+      <c r="FO3">
+        <f>FN3-FM3</f>
+        <v/>
+      </c>
+      <c r="FP3">
+        <f>EK3</f>
+        <v/>
+      </c>
+      <c r="FQ3">
+        <f>EK3</f>
+        <v/>
+      </c>
+      <c r="FR3">
+        <f>EQ3+FJ3</f>
+        <v/>
+      </c>
+      <c r="FS3">
+        <f>ER3-FJ3</f>
+        <v/>
+      </c>
+      <c r="FT3">
+        <f>DW3</f>
+        <v/>
+      </c>
+      <c r="FU3">
+        <f>FJ3</f>
+        <v/>
+      </c>
+      <c r="FV3">
+        <f>EQ3</f>
+        <v/>
+      </c>
+      <c r="FW3">
+        <f>FF3</f>
+        <v/>
+      </c>
+      <c r="FX3">
+        <f>EK3+AP3</f>
+        <v/>
+      </c>
+      <c r="FY3">
+        <f>FK3+FB3</f>
+        <v/>
+      </c>
+      <c r="FZ3">
+        <f>FL3</f>
+        <v/>
+      </c>
+      <c r="GA3">
+        <f>FF3</f>
+        <v/>
+      </c>
+      <c r="GB3">
+        <f>EK3</f>
+        <v/>
+      </c>
+      <c r="GC3">
+        <f>FK3</f>
+        <v/>
+      </c>
+      <c r="GD3">
+        <f>FB3</f>
+        <v/>
+      </c>
+      <c r="GE3">
+        <f>AP3</f>
+        <v/>
+      </c>
+      <c r="GF3">
+        <f>EK3-FK3</f>
+        <v/>
+      </c>
+      <c r="GG3">
+        <f>-FB3</f>
+        <v/>
+      </c>
+      <c r="GH3">
+        <f>FL3-FF3</f>
+        <v/>
+      </c>
+      <c r="GI3">
+        <f>FL3</f>
+        <v/>
+      </c>
+      <c r="GJ3">
+        <f>FL3</f>
+        <v/>
+      </c>
+      <c r="GK3">
+        <f>FO3</f>
+        <v/>
+      </c>
+      <c r="GL3">
+        <f>FE3</f>
+        <v/>
+      </c>
+      <c r="GM3">
+        <f>FL3+FO3+FE3</f>
+        <v/>
+      </c>
+      <c r="GN3">
+        <f>AS3</f>
+        <v/>
+      </c>
+      <c r="GO3">
+        <f>FL3+FO3+FE3-AS3</f>
+        <v/>
+      </c>
+      <c r="GP3">
+        <f>FL3+FO3+FE3</f>
+        <v/>
+      </c>
+      <c r="GQ3">
+        <f>AP3</f>
+        <v/>
+      </c>
+      <c r="GR3">
+        <f>AR3</f>
+        <v/>
+      </c>
+      <c r="GS3">
+        <f>AS3</f>
+        <v/>
+      </c>
+      <c r="GT3">
+        <f>AT3</f>
+        <v/>
+      </c>
+      <c r="GU3">
+        <f>FI3</f>
+        <v/>
+      </c>
+      <c r="GV3">
+        <f>FJ3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
@@ -7144,6 +7766,197 @@
       </c>
       <c r="EZ4" s="0">
         <f>AND(K4=0,AF4&lt;5)</f>
+        <v/>
+      </c>
+      <c r="FA4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB4">
+        <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC4">
+        <f>0*2500+0*3500+0*1200+0*300</f>
+        <v/>
+      </c>
+      <c r="FD4">
+        <f>(CF4*25+CH4*45+CJ4*80+CL4*4+CN4*9+CP4*2+CR4*4+CT4*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FE4">
+        <f>(DC4*25+DE4*45+DG4*80+DJ4*4+DL4*9+DO4*2+DQ4*4+DS4*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FF4">
+        <f>FL2</f>
+        <v/>
+      </c>
+      <c r="FG4">
+        <f>(1+AR4/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH4">
+        <f>AS2*FI2+AP4*FG4</f>
+        <v/>
+      </c>
+      <c r="FI4">
+        <f>IFERROR(FH4/(AS2+AP4),0)</f>
+        <v/>
+      </c>
+      <c r="FJ4">
+        <f>FH4*1</f>
+        <v/>
+      </c>
+      <c r="FK4">
+        <f>EQ4-DW4-DU4+FD4+FJ4</f>
+        <v/>
+      </c>
+      <c r="FL4">
+        <f>FF4+EK4+AP4-FK4-FB4</f>
+        <v/>
+      </c>
+      <c r="FM4">
+        <f>FM2+DW4</f>
+        <v/>
+      </c>
+      <c r="FN4">
+        <f>FN2+FC4</f>
+        <v/>
+      </c>
+      <c r="FO4">
+        <f>FN4-FM4</f>
+        <v/>
+      </c>
+      <c r="FP4">
+        <f>EK4</f>
+        <v/>
+      </c>
+      <c r="FQ4">
+        <f>EK4</f>
+        <v/>
+      </c>
+      <c r="FR4">
+        <f>EQ4+FJ4</f>
+        <v/>
+      </c>
+      <c r="FS4">
+        <f>ER4-FJ4</f>
+        <v/>
+      </c>
+      <c r="FT4">
+        <f>DW4</f>
+        <v/>
+      </c>
+      <c r="FU4">
+        <f>FJ4</f>
+        <v/>
+      </c>
+      <c r="FV4">
+        <f>EQ4</f>
+        <v/>
+      </c>
+      <c r="FW4">
+        <f>FF4</f>
+        <v/>
+      </c>
+      <c r="FX4">
+        <f>EK4+AP4</f>
+        <v/>
+      </c>
+      <c r="FY4">
+        <f>FK4+FB4</f>
+        <v/>
+      </c>
+      <c r="FZ4">
+        <f>FL4</f>
+        <v/>
+      </c>
+      <c r="GA4">
+        <f>FF4</f>
+        <v/>
+      </c>
+      <c r="GB4">
+        <f>EK4</f>
+        <v/>
+      </c>
+      <c r="GC4">
+        <f>FK4</f>
+        <v/>
+      </c>
+      <c r="GD4">
+        <f>FB4</f>
+        <v/>
+      </c>
+      <c r="GE4">
+        <f>AP4</f>
+        <v/>
+      </c>
+      <c r="GF4">
+        <f>EK4-FK4</f>
+        <v/>
+      </c>
+      <c r="GG4">
+        <f>-FB4</f>
+        <v/>
+      </c>
+      <c r="GH4">
+        <f>FL4-FF4</f>
+        <v/>
+      </c>
+      <c r="GI4">
+        <f>FL4</f>
+        <v/>
+      </c>
+      <c r="GJ4">
+        <f>FL4</f>
+        <v/>
+      </c>
+      <c r="GK4">
+        <f>FO4</f>
+        <v/>
+      </c>
+      <c r="GL4">
+        <f>FE4</f>
+        <v/>
+      </c>
+      <c r="GM4">
+        <f>FL4+FO4+FE4</f>
+        <v/>
+      </c>
+      <c r="GN4">
+        <f>AS4</f>
+        <v/>
+      </c>
+      <c r="GO4">
+        <f>FL4+FO4+FE4-AS4</f>
+        <v/>
+      </c>
+      <c r="GP4">
+        <f>FL4+FO4+FE4</f>
+        <v/>
+      </c>
+      <c r="GQ4">
+        <f>AP4</f>
+        <v/>
+      </c>
+      <c r="GR4">
+        <f>AR4</f>
+        <v/>
+      </c>
+      <c r="GS4">
+        <f>AS4</f>
+        <v/>
+      </c>
+      <c r="GT4">
+        <f>AT4</f>
+        <v/>
+      </c>
+      <c r="GU4">
+        <f>FI4</f>
+        <v/>
+      </c>
+      <c r="GV4">
+        <f>FJ4</f>
         <v/>
       </c>
     </row>
@@ -7722,6 +8535,197 @@
         <f>AND(K5=0,AF5&lt;5)</f>
         <v/>
       </c>
+      <c r="FA5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB5">
+        <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC5">
+        <f>0*2500+0*3500+0*1200+0*300</f>
+        <v/>
+      </c>
+      <c r="FD5">
+        <f>(CF5*25+CH5*45+CJ5*80+CL5*4+CN5*9+CP5*2+CR5*4+CT5*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FE5">
+        <f>(DC5*25+DE5*45+DG5*80+DJ5*4+DL5*9+DO5*2+DQ5*4+DS5*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF5">
+        <f>FL3</f>
+        <v/>
+      </c>
+      <c r="FG5">
+        <f>(1+AR5/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH5">
+        <f>AS3*FI3+AP5*FG5</f>
+        <v/>
+      </c>
+      <c r="FI5">
+        <f>IFERROR(FH5/(AS3+AP5),0)</f>
+        <v/>
+      </c>
+      <c r="FJ5">
+        <f>FH5*1</f>
+        <v/>
+      </c>
+      <c r="FK5">
+        <f>EQ5-DW5-DU5+FD5+FJ5</f>
+        <v/>
+      </c>
+      <c r="FL5">
+        <f>FF5+EK5+AP5-FK5-FB5</f>
+        <v/>
+      </c>
+      <c r="FM5">
+        <f>FM3+DW5</f>
+        <v/>
+      </c>
+      <c r="FN5">
+        <f>FN3+FC5</f>
+        <v/>
+      </c>
+      <c r="FO5">
+        <f>FN5-FM5</f>
+        <v/>
+      </c>
+      <c r="FP5">
+        <f>EK5</f>
+        <v/>
+      </c>
+      <c r="FQ5">
+        <f>EK5</f>
+        <v/>
+      </c>
+      <c r="FR5">
+        <f>EQ5+FJ5</f>
+        <v/>
+      </c>
+      <c r="FS5">
+        <f>ER5-FJ5</f>
+        <v/>
+      </c>
+      <c r="FT5">
+        <f>DW5</f>
+        <v/>
+      </c>
+      <c r="FU5">
+        <f>FJ5</f>
+        <v/>
+      </c>
+      <c r="FV5">
+        <f>EQ5</f>
+        <v/>
+      </c>
+      <c r="FW5">
+        <f>FF5</f>
+        <v/>
+      </c>
+      <c r="FX5">
+        <f>EK5+AP5</f>
+        <v/>
+      </c>
+      <c r="FY5">
+        <f>FK5+FB5</f>
+        <v/>
+      </c>
+      <c r="FZ5">
+        <f>FL5</f>
+        <v/>
+      </c>
+      <c r="GA5">
+        <f>FF5</f>
+        <v/>
+      </c>
+      <c r="GB5">
+        <f>EK5</f>
+        <v/>
+      </c>
+      <c r="GC5">
+        <f>FK5</f>
+        <v/>
+      </c>
+      <c r="GD5">
+        <f>FB5</f>
+        <v/>
+      </c>
+      <c r="GE5">
+        <f>AP5</f>
+        <v/>
+      </c>
+      <c r="GF5">
+        <f>EK5-FK5</f>
+        <v/>
+      </c>
+      <c r="GG5">
+        <f>-FB5</f>
+        <v/>
+      </c>
+      <c r="GH5">
+        <f>FL5-FF5</f>
+        <v/>
+      </c>
+      <c r="GI5">
+        <f>FL5</f>
+        <v/>
+      </c>
+      <c r="GJ5">
+        <f>FL5</f>
+        <v/>
+      </c>
+      <c r="GK5">
+        <f>FO5</f>
+        <v/>
+      </c>
+      <c r="GL5">
+        <f>FE5</f>
+        <v/>
+      </c>
+      <c r="GM5">
+        <f>FL5+FO5+FE5</f>
+        <v/>
+      </c>
+      <c r="GN5">
+        <f>AS5</f>
+        <v/>
+      </c>
+      <c r="GO5">
+        <f>FL5+FO5+FE5-AS5</f>
+        <v/>
+      </c>
+      <c r="GP5">
+        <f>FL5+FO5+FE5</f>
+        <v/>
+      </c>
+      <c r="GQ5">
+        <f>AP5</f>
+        <v/>
+      </c>
+      <c r="GR5">
+        <f>AR5</f>
+        <v/>
+      </c>
+      <c r="GS5">
+        <f>AS5</f>
+        <v/>
+      </c>
+      <c r="GT5">
+        <f>AT5</f>
+        <v/>
+      </c>
+      <c r="GU5">
+        <f>FI5</f>
+        <v/>
+      </c>
+      <c r="GV5">
+        <f>FJ5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="n">
@@ -8312,6 +9316,197 @@
       </c>
       <c r="EZ6" s="0">
         <f>AND(K6=0,AF6&lt;5)</f>
+        <v/>
+      </c>
+      <c r="FA6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB6">
+        <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC6">
+        <f>0*2500+0*3500+0*1200+0*300</f>
+        <v/>
+      </c>
+      <c r="FD6">
+        <f>(CF6*25+CH6*45+CJ6*80+CL6*4+CN6*9+CP6*2+CR6*4+CT6*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FE6">
+        <f>(DC6*25+DE6*45+DG6*80+DJ6*4+DL6*9+DO6*2+DQ6*4+DS6*7)*0.8924</f>
+        <v/>
+      </c>
+      <c r="FF6">
+        <f>FL4</f>
+        <v/>
+      </c>
+      <c r="FG6">
+        <f>(1+AR6/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH6">
+        <f>AS4*FI4+AP6*FG6</f>
+        <v/>
+      </c>
+      <c r="FI6">
+        <f>IFERROR(FH6/(AS4+AP6),0)</f>
+        <v/>
+      </c>
+      <c r="FJ6">
+        <f>FH6*1</f>
+        <v/>
+      </c>
+      <c r="FK6">
+        <f>EQ6-DW6-DU6+FD6+FJ6</f>
+        <v/>
+      </c>
+      <c r="FL6">
+        <f>FF6+EK6+AP6-FK6-FB6</f>
+        <v/>
+      </c>
+      <c r="FM6">
+        <f>FM4+DW6</f>
+        <v/>
+      </c>
+      <c r="FN6">
+        <f>FN4+FC6</f>
+        <v/>
+      </c>
+      <c r="FO6">
+        <f>FN6-FM6</f>
+        <v/>
+      </c>
+      <c r="FP6">
+        <f>EK6</f>
+        <v/>
+      </c>
+      <c r="FQ6">
+        <f>EK6</f>
+        <v/>
+      </c>
+      <c r="FR6">
+        <f>EQ6+FJ6</f>
+        <v/>
+      </c>
+      <c r="FS6">
+        <f>ER6-FJ6</f>
+        <v/>
+      </c>
+      <c r="FT6">
+        <f>DW6</f>
+        <v/>
+      </c>
+      <c r="FU6">
+        <f>FJ6</f>
+        <v/>
+      </c>
+      <c r="FV6">
+        <f>EQ6</f>
+        <v/>
+      </c>
+      <c r="FW6">
+        <f>FF6</f>
+        <v/>
+      </c>
+      <c r="FX6">
+        <f>EK6+AP6</f>
+        <v/>
+      </c>
+      <c r="FY6">
+        <f>FK6+FB6</f>
+        <v/>
+      </c>
+      <c r="FZ6">
+        <f>FL6</f>
+        <v/>
+      </c>
+      <c r="GA6">
+        <f>FF6</f>
+        <v/>
+      </c>
+      <c r="GB6">
+        <f>EK6</f>
+        <v/>
+      </c>
+      <c r="GC6">
+        <f>FK6</f>
+        <v/>
+      </c>
+      <c r="GD6">
+        <f>FB6</f>
+        <v/>
+      </c>
+      <c r="GE6">
+        <f>AP6</f>
+        <v/>
+      </c>
+      <c r="GF6">
+        <f>EK6-FK6</f>
+        <v/>
+      </c>
+      <c r="GG6">
+        <f>-FB6</f>
+        <v/>
+      </c>
+      <c r="GH6">
+        <f>FL6-FF6</f>
+        <v/>
+      </c>
+      <c r="GI6">
+        <f>FL6</f>
+        <v/>
+      </c>
+      <c r="GJ6">
+        <f>FL6</f>
+        <v/>
+      </c>
+      <c r="GK6">
+        <f>FO6</f>
+        <v/>
+      </c>
+      <c r="GL6">
+        <f>FE6</f>
+        <v/>
+      </c>
+      <c r="GM6">
+        <f>FL6+FO6+FE6</f>
+        <v/>
+      </c>
+      <c r="GN6">
+        <f>AS6</f>
+        <v/>
+      </c>
+      <c r="GO6">
+        <f>FL6+FO6+FE6-AS6</f>
+        <v/>
+      </c>
+      <c r="GP6">
+        <f>FL6+FO6+FE6</f>
+        <v/>
+      </c>
+      <c r="GQ6">
+        <f>AP6</f>
+        <v/>
+      </c>
+      <c r="GR6">
+        <f>AR6</f>
+        <v/>
+      </c>
+      <c r="GS6">
+        <f>AS6</f>
+        <v/>
+      </c>
+      <c r="GT6">
+        <f>AT6</f>
+        <v/>
+      </c>
+      <c r="GU6">
+        <f>FI6</f>
+        <v/>
+      </c>
+      <c r="GV6">
+        <f>FJ6</f>
         <v/>
       </c>
     </row>
@@ -8896,6 +10091,197 @@
       </c>
       <c r="EZ7" s="0">
         <f>AND(K7=0,AF7&lt;5)</f>
+        <v/>
+      </c>
+      <c r="FA7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="FB7">
+        <f>0*2500*(1+0.03+0.02)+0*3500*(1+0.03+0.02)+0*1200*(1+0.03+0.02)+0*300*(1+0+0.01)</f>
+        <v/>
+      </c>
+      <c r="FC7">
+        <f>0*2500+0*3500+0*1200+0*300</f>
+        <v/>
+      </c>
+      <c r="FD7">
+        <f>(CF7*25+CH7*45+CJ7*80+CL7*4+CN7*9+CP7*2+CR7*4+CT7*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FE7">
+        <f>(DC7*25+DE7*45+DG7*80+DJ7*4+DL7*9+DO7*2+DQ7*4+DS7*7)*0.92</f>
+        <v/>
+      </c>
+      <c r="FF7">
+        <f>FL5</f>
+        <v/>
+      </c>
+      <c r="FG7">
+        <f>(1+AR7/100)^(1/12)-1</f>
+        <v/>
+      </c>
+      <c r="FH7">
+        <f>AS5*FI5+AP7*FG7</f>
+        <v/>
+      </c>
+      <c r="FI7">
+        <f>IFERROR(FH7/(AS5+AP7),0)</f>
+        <v/>
+      </c>
+      <c r="FJ7">
+        <f>FH7*1</f>
+        <v/>
+      </c>
+      <c r="FK7">
+        <f>EQ7-DW7-DU7+FD7+FJ7</f>
+        <v/>
+      </c>
+      <c r="FL7">
+        <f>FF7+EK7+AP7-FK7-FB7</f>
+        <v/>
+      </c>
+      <c r="FM7">
+        <f>FM5+DW7</f>
+        <v/>
+      </c>
+      <c r="FN7">
+        <f>FN5+FC7</f>
+        <v/>
+      </c>
+      <c r="FO7">
+        <f>FN7-FM7</f>
+        <v/>
+      </c>
+      <c r="FP7">
+        <f>EK7</f>
+        <v/>
+      </c>
+      <c r="FQ7">
+        <f>EK7</f>
+        <v/>
+      </c>
+      <c r="FR7">
+        <f>EQ7+FJ7</f>
+        <v/>
+      </c>
+      <c r="FS7">
+        <f>ER7-FJ7</f>
+        <v/>
+      </c>
+      <c r="FT7">
+        <f>DW7</f>
+        <v/>
+      </c>
+      <c r="FU7">
+        <f>FJ7</f>
+        <v/>
+      </c>
+      <c r="FV7">
+        <f>EQ7</f>
+        <v/>
+      </c>
+      <c r="FW7">
+        <f>FF7</f>
+        <v/>
+      </c>
+      <c r="FX7">
+        <f>EK7+AP7</f>
+        <v/>
+      </c>
+      <c r="FY7">
+        <f>FK7+FB7</f>
+        <v/>
+      </c>
+      <c r="FZ7">
+        <f>FL7</f>
+        <v/>
+      </c>
+      <c r="GA7">
+        <f>FF7</f>
+        <v/>
+      </c>
+      <c r="GB7">
+        <f>EK7</f>
+        <v/>
+      </c>
+      <c r="GC7">
+        <f>FK7</f>
+        <v/>
+      </c>
+      <c r="GD7">
+        <f>FB7</f>
+        <v/>
+      </c>
+      <c r="GE7">
+        <f>AP7</f>
+        <v/>
+      </c>
+      <c r="GF7">
+        <f>EK7-FK7</f>
+        <v/>
+      </c>
+      <c r="GG7">
+        <f>-FB7</f>
+        <v/>
+      </c>
+      <c r="GH7">
+        <f>FL7-FF7</f>
+        <v/>
+      </c>
+      <c r="GI7">
+        <f>FL7</f>
+        <v/>
+      </c>
+      <c r="GJ7">
+        <f>FL7</f>
+        <v/>
+      </c>
+      <c r="GK7">
+        <f>FO7</f>
+        <v/>
+      </c>
+      <c r="GL7">
+        <f>FE7</f>
+        <v/>
+      </c>
+      <c r="GM7">
+        <f>FL7+FO7+FE7</f>
+        <v/>
+      </c>
+      <c r="GN7">
+        <f>AS7</f>
+        <v/>
+      </c>
+      <c r="GO7">
+        <f>FL7+FO7+FE7-AS7</f>
+        <v/>
+      </c>
+      <c r="GP7">
+        <f>FL7+FO7+FE7</f>
+        <v/>
+      </c>
+      <c r="GQ7">
+        <f>AP7</f>
+        <v/>
+      </c>
+      <c r="GR7">
+        <f>AR7</f>
+        <v/>
+      </c>
+      <c r="GS7">
+        <f>AS7</f>
+        <v/>
+      </c>
+      <c r="GT7">
+        <f>AT7</f>
+        <v/>
+      </c>
+      <c r="GU7">
+        <f>FI7</f>
+        <v/>
+      </c>
+      <c r="GV7">
+        <f>FJ7</f>
         <v/>
       </c>
     </row>
@@ -12431,2324 +13817,2324 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>ciclo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>empresa</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>segmento</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>molde</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>cuero</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
         <is>
           <t>accesorios</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="0" t="inlineStr">
         <is>
           <t>hilo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="0" t="inlineStr">
         <is>
           <t>cantidad</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="0" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="0" t="inlineStr">
         <is>
           <t>calidad</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-01</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-02</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-03</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-04</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-05</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-06</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-07</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="0" t="inlineStr">
         <is>
           <t>disponible_INS-08</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="0" t="inlineStr">
         <is>
           <t>capacidadAsignada</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="0" t="inlineStr">
         <is>
           <t>producidoPre</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="0" t="inlineStr">
         <is>
           <t>producido</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-01</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-01</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-01</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-02</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-02</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-02</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-03</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-03</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-03</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-04</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-04</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-04</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-05</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-05</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-05</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-06</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-06</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-06</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-07</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-07</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-07</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="0" t="inlineStr">
         <is>
           <t>usadoPre_INS-08</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="0" t="inlineStr">
         <is>
           <t>saldoPre_INS-08</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="0" t="inlineStr">
         <is>
           <t>usado_INS-08</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="0" t="inlineStr">
         <is>
           <t>precioFactor</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="0" t="inlineStr">
         <is>
           <t>precioEfectivo</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="0" t="inlineStr">
         <is>
           <t>stockAntes</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="0" t="inlineStr">
         <is>
           <t>vendido</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AX1" s="0" t="inlineStr">
         <is>
           <t>ingreso</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="0" t="inlineStr">
         <is>
           <t>inventarioFinal</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>INF-10</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>INS-03</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="0" t="inlineStr">
         <is>
           <t>INS-05</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="0" t="inlineStr">
         <is>
           <t>INS-08</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E2,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F2,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G2,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D2,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K2">
+      <c r="K2" s="0">
         <f>'Pipeline_sim2'!CG2</f>
         <v/>
       </c>
-      <c r="L2">
+      <c r="L2" s="0">
         <f>'Pipeline_sim2'!CI2</f>
         <v/>
       </c>
-      <c r="M2">
+      <c r="M2" s="0">
         <f>'Pipeline_sim2'!CK2</f>
         <v/>
       </c>
-      <c r="N2">
+      <c r="N2" s="0">
         <f>'Pipeline_sim2'!CM2</f>
         <v/>
       </c>
-      <c r="O2">
+      <c r="O2" s="0">
         <f>'Pipeline_sim2'!CO2</f>
         <v/>
       </c>
-      <c r="P2">
+      <c r="P2" s="0">
         <f>'Pipeline_sim2'!CQ2</f>
         <v/>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="0">
         <f>'Pipeline_sim2'!CS2</f>
         <v/>
       </c>
-      <c r="R2">
+      <c r="R2" s="0">
         <f>'Pipeline_sim2'!CU2</f>
         <v/>
       </c>
-      <c r="S2">
+      <c r="S2" s="0">
         <f>IFERROR(ROUNDDOWN(H2*'Pipeline_sim2'!CE2/'Pipeline_sim2'!I2,0),0)</f>
         <v/>
       </c>
-      <c r="T2">
+      <c r="T2" s="0">
         <f>ROUNDDOWN(MIN(H2,S2,(M2)/0.7,(O2)/1,(R2)/13),0)</f>
         <v/>
       </c>
-      <c r="U2">
+      <c r="U2" s="0">
         <f>ROUNDDOWN(T2*'Pipeline_sim2'!AU2,0)</f>
         <v/>
       </c>
-      <c r="V2">
+      <c r="V2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="W2">
+      <c r="W2" s="0">
         <f>K2-V2</f>
         <v/>
       </c>
-      <c r="X2">
+      <c r="X2" s="0">
         <f>IFERROR(V2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="Y2">
+      <c r="Y2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z2">
+      <c r="Z2" s="0">
         <f>L2-Y2</f>
         <v/>
       </c>
-      <c r="AA2">
+      <c r="AA2" s="0">
         <f>IFERROR(Y2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AB2">
+      <c r="AB2" s="0">
         <f>MIN(M2,MAX(0,T2*0.7-(V2+Y2)))</f>
         <v/>
       </c>
-      <c r="AC2">
+      <c r="AC2" s="0">
         <f>M2-AB2</f>
         <v/>
       </c>
-      <c r="AD2">
+      <c r="AD2" s="0">
         <f>IFERROR(AB2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AE2">
+      <c r="AE2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AF2">
+      <c r="AF2" s="0">
         <f>N2-AE2</f>
         <v/>
       </c>
-      <c r="AG2">
+      <c r="AG2" s="0">
         <f>IFERROR(AE2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AH2">
+      <c r="AH2" s="0">
         <f>MIN(O2,MAX(0,T2*1-(AE2)))</f>
         <v/>
       </c>
-      <c r="AI2">
+      <c r="AI2" s="0">
         <f>O2-AH2</f>
         <v/>
       </c>
-      <c r="AJ2">
+      <c r="AJ2" s="0">
         <f>IFERROR(AH2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AK2">
+      <c r="AK2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AL2">
+      <c r="AL2" s="0">
         <f>P2-AK2</f>
         <v/>
       </c>
-      <c r="AM2">
+      <c r="AM2" s="0">
         <f>IFERROR(AK2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AN2">
+      <c r="AN2" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO2">
+      <c r="AO2" s="0">
         <f>Q2-AN2</f>
         <v/>
       </c>
-      <c r="AP2">
+      <c r="AP2" s="0">
         <f>IFERROR(AN2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AQ2">
+      <c r="AQ2" s="0">
         <f>MIN(R2,MAX(0,T2*13-(AK2+AN2)))</f>
         <v/>
       </c>
-      <c r="AR2">
+      <c r="AR2" s="0">
         <f>R2-AQ2</f>
         <v/>
       </c>
-      <c r="AS2">
+      <c r="AS2" s="0">
         <f>IFERROR(AQ2*U2/T2,0)</f>
         <v/>
       </c>
-      <c r="AT2">
+      <c r="AT2" s="0">
         <f>IF(AND(C2="SEG-03",H2&gt;0),IF(J2&lt;4,0.65,IF(J2&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU2">
+      <c r="AU2" s="0">
         <f>I2*AT2</f>
         <v/>
       </c>
-      <c r="AV2">
+      <c r="AV2" s="0">
         <f>0+U2</f>
         <v/>
       </c>
-      <c r="AW2">
+      <c r="AW2" s="0">
         <f>MIN(AV2,MAX(0,'Mercados_Pipeline_sim2'!I2))</f>
         <v/>
       </c>
-      <c r="AX2">
+      <c r="AX2" s="0">
         <f>AW2*AU2</f>
         <v/>
       </c>
-      <c r="AY2">
+      <c r="AY2" s="0">
         <f>AV2-AW2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="F3" s="0" t="inlineStr"/>
+      <c r="G3" s="0" t="inlineStr"/>
+      <c r="H3" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E3,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F3,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G3,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D3,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K3">
+      <c r="K3" s="0">
         <f>'Pipeline_sim2'!CG3</f>
         <v/>
       </c>
-      <c r="L3">
+      <c r="L3" s="0">
         <f>'Pipeline_sim2'!CI3</f>
         <v/>
       </c>
-      <c r="M3">
+      <c r="M3" s="0">
         <f>'Pipeline_sim2'!CK3</f>
         <v/>
       </c>
-      <c r="N3">
+      <c r="N3" s="0">
         <f>'Pipeline_sim2'!CM3</f>
         <v/>
       </c>
-      <c r="O3">
+      <c r="O3" s="0">
         <f>'Pipeline_sim2'!CO3</f>
         <v/>
       </c>
-      <c r="P3">
+      <c r="P3" s="0">
         <f>'Pipeline_sim2'!CQ3</f>
         <v/>
       </c>
-      <c r="Q3">
+      <c r="Q3" s="0">
         <f>'Pipeline_sim2'!CS3</f>
         <v/>
       </c>
-      <c r="R3">
+      <c r="R3" s="0">
         <f>'Pipeline_sim2'!CU3</f>
         <v/>
       </c>
-      <c r="S3">
+      <c r="S3" s="0">
         <f>IFERROR(ROUNDDOWN(H3*'Pipeline_sim2'!CE3/'Pipeline_sim2'!I3,0),0)</f>
         <v/>
       </c>
-      <c r="T3">
+      <c r="T3" s="0">
         <f>ROUNDDOWN(MIN(H3,S3,(K3)/0.3,(N3+O3)/1,(P3+Q3+R3)/6),0)</f>
         <v/>
       </c>
-      <c r="U3">
+      <c r="U3" s="0">
         <f>ROUNDDOWN(T3*'Pipeline_sim2'!AU3,0)</f>
         <v/>
       </c>
-      <c r="V3">
+      <c r="V3" s="0">
         <f>MIN(K3,MAX(0,T3*0.3))</f>
         <v/>
       </c>
-      <c r="W3">
+      <c r="W3" s="0">
         <f>K3-V3</f>
         <v/>
       </c>
-      <c r="X3">
+      <c r="X3" s="0">
         <f>IFERROR(V3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="Y3">
+      <c r="Y3" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z3">
+      <c r="Z3" s="0">
         <f>L3-Y3</f>
         <v/>
       </c>
-      <c r="AA3">
+      <c r="AA3" s="0">
         <f>IFERROR(Y3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AB3">
+      <c r="AB3" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC3">
+      <c r="AC3" s="0">
         <f>M3-AB3</f>
         <v/>
       </c>
-      <c r="AD3">
+      <c r="AD3" s="0">
         <f>IFERROR(AB3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AE3">
+      <c r="AE3" s="0">
         <f>MIN(N3,MAX(0,T3*1))</f>
         <v/>
       </c>
-      <c r="AF3">
+      <c r="AF3" s="0">
         <f>N3-AE3</f>
         <v/>
       </c>
-      <c r="AG3">
+      <c r="AG3" s="0">
         <f>IFERROR(AE3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AH3">
+      <c r="AH3" s="0">
         <f>MIN(O3,MAX(0,T3*1-(AE3)))</f>
         <v/>
       </c>
-      <c r="AI3">
+      <c r="AI3" s="0">
         <f>O3-AH3</f>
         <v/>
       </c>
-      <c r="AJ3">
+      <c r="AJ3" s="0">
         <f>IFERROR(AH3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AK3">
+      <c r="AK3" s="0">
         <f>MIN(P3,MAX(0,T3*6))</f>
         <v/>
       </c>
-      <c r="AL3">
+      <c r="AL3" s="0">
         <f>P3-AK3</f>
         <v/>
       </c>
-      <c r="AM3">
+      <c r="AM3" s="0">
         <f>IFERROR(AK3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AN3">
+      <c r="AN3" s="0">
         <f>MIN(Q3,MAX(0,T3*6-(AK3)))</f>
         <v/>
       </c>
-      <c r="AO3">
+      <c r="AO3" s="0">
         <f>Q3-AN3</f>
         <v/>
       </c>
-      <c r="AP3">
+      <c r="AP3" s="0">
         <f>IFERROR(AN3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AQ3">
+      <c r="AQ3" s="0">
         <f>MIN(R3,MAX(0,T3*6-(AK3+AN3)))</f>
         <v/>
       </c>
-      <c r="AR3">
+      <c r="AR3" s="0">
         <f>R3-AQ3</f>
         <v/>
       </c>
-      <c r="AS3">
+      <c r="AS3" s="0">
         <f>IFERROR(AQ3*U3/T3,0)</f>
         <v/>
       </c>
-      <c r="AT3">
+      <c r="AT3" s="0">
         <f>IF(AND(C3="SEG-03",H3&gt;0),IF(J3&lt;4,0.65,IF(J3&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU3">
+      <c r="AU3" s="0">
         <f>I3*AT3</f>
         <v/>
       </c>
-      <c r="AV3">
+      <c r="AV3" s="0">
         <f>0+U3</f>
         <v/>
       </c>
-      <c r="AW3">
+      <c r="AW3" s="0">
         <f>MIN(AV3,MAX(0,'Mercados_Pipeline_sim2'!I3))</f>
         <v/>
       </c>
-      <c r="AX3">
+      <c r="AX3" s="0">
         <f>AW3*AU3</f>
         <v/>
       </c>
-      <c r="AY3">
+      <c r="AY3" s="0">
         <f>AV3-AW3</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="0" t="inlineStr">
         <is>
           <t>INS-04</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>INS-06</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E4,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F4,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G4,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D4,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K4">
+      <c r="K4" s="0">
         <f>'Lotes_Pipeline_sim2'!W3</f>
         <v/>
       </c>
-      <c r="L4">
+      <c r="L4" s="0">
         <f>'Lotes_Pipeline_sim2'!Z3</f>
         <v/>
       </c>
-      <c r="M4">
+      <c r="M4" s="0">
         <f>'Lotes_Pipeline_sim2'!AC3</f>
         <v/>
       </c>
-      <c r="N4">
+      <c r="N4" s="0">
         <f>'Lotes_Pipeline_sim2'!AF3</f>
         <v/>
       </c>
-      <c r="O4">
+      <c r="O4" s="0">
         <f>'Lotes_Pipeline_sim2'!AI3</f>
         <v/>
       </c>
-      <c r="P4">
+      <c r="P4" s="0">
         <f>'Lotes_Pipeline_sim2'!AL3</f>
         <v/>
       </c>
-      <c r="Q4">
+      <c r="Q4" s="0">
         <f>'Lotes_Pipeline_sim2'!AO3</f>
         <v/>
       </c>
-      <c r="R4">
+      <c r="R4" s="0">
         <f>'Lotes_Pipeline_sim2'!AR3</f>
         <v/>
       </c>
-      <c r="S4">
+      <c r="S4" s="0">
         <f>IFERROR(ROUNDDOWN(H4*'Pipeline_sim2'!CE3/'Pipeline_sim2'!I3,0),0)</f>
         <v/>
       </c>
-      <c r="T4">
+      <c r="T4" s="0">
         <f>ROUNDDOWN(MIN(H4,S4,(K4)/0.3,(N4)/1,(P4)/6),0)</f>
         <v/>
       </c>
-      <c r="U4">
+      <c r="U4" s="0">
         <f>ROUNDDOWN(T4*'Pipeline_sim2'!AU3,0)</f>
         <v/>
       </c>
-      <c r="V4">
+      <c r="V4" s="0">
         <f>MIN(K4,MAX(0,T4*0.3))</f>
         <v/>
       </c>
-      <c r="W4">
+      <c r="W4" s="0">
         <f>K4-V4</f>
         <v/>
       </c>
-      <c r="X4">
+      <c r="X4" s="0">
         <f>IFERROR(V4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="Y4">
+      <c r="Y4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z4">
+      <c r="Z4" s="0">
         <f>L4-Y4</f>
         <v/>
       </c>
-      <c r="AA4">
+      <c r="AA4" s="0">
         <f>IFERROR(Y4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AB4">
+      <c r="AB4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC4">
+      <c r="AC4" s="0">
         <f>M4-AB4</f>
         <v/>
       </c>
-      <c r="AD4">
+      <c r="AD4" s="0">
         <f>IFERROR(AB4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AE4">
+      <c r="AE4" s="0">
         <f>MIN(N4,MAX(0,T4*1))</f>
         <v/>
       </c>
-      <c r="AF4">
+      <c r="AF4" s="0">
         <f>N4-AE4</f>
         <v/>
       </c>
-      <c r="AG4">
+      <c r="AG4" s="0">
         <f>IFERROR(AE4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AH4">
+      <c r="AH4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AI4">
+      <c r="AI4" s="0">
         <f>O4-AH4</f>
         <v/>
       </c>
-      <c r="AJ4">
+      <c r="AJ4" s="0">
         <f>IFERROR(AH4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AK4">
+      <c r="AK4" s="0">
         <f>MIN(P4,MAX(0,T4*6))</f>
         <v/>
       </c>
-      <c r="AL4">
+      <c r="AL4" s="0">
         <f>P4-AK4</f>
         <v/>
       </c>
-      <c r="AM4">
+      <c r="AM4" s="0">
         <f>IFERROR(AK4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AN4">
+      <c r="AN4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO4">
+      <c r="AO4" s="0">
         <f>Q4-AN4</f>
         <v/>
       </c>
-      <c r="AP4">
+      <c r="AP4" s="0">
         <f>IFERROR(AN4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AQ4">
+      <c r="AQ4" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AR4">
+      <c r="AR4" s="0">
         <f>R4-AQ4</f>
         <v/>
       </c>
-      <c r="AS4">
+      <c r="AS4" s="0">
         <f>IFERROR(AQ4*U4/T4,0)</f>
         <v/>
       </c>
-      <c r="AT4">
+      <c r="AT4" s="0">
         <f>IF(AND(C4="SEG-03",H4&gt;0),IF(J4&lt;4,0.65,IF(J4&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU4">
+      <c r="AU4" s="0">
         <f>I4*AT4</f>
         <v/>
       </c>
-      <c r="AV4">
+      <c r="AV4" s="0">
         <f>0+U4</f>
         <v/>
       </c>
-      <c r="AW4">
+      <c r="AW4" s="0">
         <f>MIN(AV4,MAX(0,'Mercados_Pipeline_sim2'!I3-('Lotes_Pipeline_sim2'!AW3)))</f>
         <v/>
       </c>
-      <c r="AX4">
+      <c r="AX4" s="0">
         <f>AW4*AU4</f>
         <v/>
       </c>
-      <c r="AY4">
+      <c r="AY4" s="0">
         <f>AV4-AW4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>INF-10</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>INS-03</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>INS-05</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>INS-08</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E5,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F5,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G5,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D5,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K5">
+      <c r="K5" s="0">
         <f>'Pipeline_sim2'!CG4</f>
         <v/>
       </c>
-      <c r="L5">
+      <c r="L5" s="0">
         <f>'Pipeline_sim2'!CI4</f>
         <v/>
       </c>
-      <c r="M5">
+      <c r="M5" s="0">
         <f>'Pipeline_sim2'!CK4</f>
         <v/>
       </c>
-      <c r="N5">
+      <c r="N5" s="0">
         <f>'Pipeline_sim2'!CM4</f>
         <v/>
       </c>
-      <c r="O5">
+      <c r="O5" s="0">
         <f>'Pipeline_sim2'!CO4</f>
         <v/>
       </c>
-      <c r="P5">
+      <c r="P5" s="0">
         <f>'Pipeline_sim2'!CQ4</f>
         <v/>
       </c>
-      <c r="Q5">
+      <c r="Q5" s="0">
         <f>'Pipeline_sim2'!CS4</f>
         <v/>
       </c>
-      <c r="R5">
+      <c r="R5" s="0">
         <f>'Pipeline_sim2'!CU4</f>
         <v/>
       </c>
-      <c r="S5">
+      <c r="S5" s="0">
         <f>IFERROR(ROUNDDOWN(H5*'Pipeline_sim2'!CE4/'Pipeline_sim2'!I4,0),0)</f>
         <v/>
       </c>
-      <c r="T5">
+      <c r="T5" s="0">
         <f>ROUNDDOWN(MIN(H5,S5,(M5)/0.7,(O5)/1,(R5)/13),0)</f>
         <v/>
       </c>
-      <c r="U5">
+      <c r="U5" s="0">
         <f>ROUNDDOWN(T5*'Pipeline_sim2'!AU4,0)</f>
         <v/>
       </c>
-      <c r="V5">
+      <c r="V5" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="W5">
+      <c r="W5" s="0">
         <f>K5-V5</f>
         <v/>
       </c>
-      <c r="X5">
+      <c r="X5" s="0">
         <f>IFERROR(V5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="Y5">
+      <c r="Y5" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z5">
+      <c r="Z5" s="0">
         <f>L5-Y5</f>
         <v/>
       </c>
-      <c r="AA5">
+      <c r="AA5" s="0">
         <f>IFERROR(Y5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AB5">
+      <c r="AB5" s="0">
         <f>MIN(M5,MAX(0,T5*0.7-(V5+Y5)))</f>
         <v/>
       </c>
-      <c r="AC5">
+      <c r="AC5" s="0">
         <f>M5-AB5</f>
         <v/>
       </c>
-      <c r="AD5">
+      <c r="AD5" s="0">
         <f>IFERROR(AB5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AE5">
+      <c r="AE5" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AF5">
+      <c r="AF5" s="0">
         <f>N5-AE5</f>
         <v/>
       </c>
-      <c r="AG5">
+      <c r="AG5" s="0">
         <f>IFERROR(AE5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AH5">
+      <c r="AH5" s="0">
         <f>MIN(O5,MAX(0,T5*1-(AE5)))</f>
         <v/>
       </c>
-      <c r="AI5">
+      <c r="AI5" s="0">
         <f>O5-AH5</f>
         <v/>
       </c>
-      <c r="AJ5">
+      <c r="AJ5" s="0">
         <f>IFERROR(AH5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AK5">
+      <c r="AK5" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AL5">
+      <c r="AL5" s="0">
         <f>P5-AK5</f>
         <v/>
       </c>
-      <c r="AM5">
+      <c r="AM5" s="0">
         <f>IFERROR(AK5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AN5">
+      <c r="AN5" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO5">
+      <c r="AO5" s="0">
         <f>Q5-AN5</f>
         <v/>
       </c>
-      <c r="AP5">
+      <c r="AP5" s="0">
         <f>IFERROR(AN5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AQ5">
+      <c r="AQ5" s="0">
         <f>MIN(R5,MAX(0,T5*13-(AK5+AN5)))</f>
         <v/>
       </c>
-      <c r="AR5">
+      <c r="AR5" s="0">
         <f>R5-AQ5</f>
         <v/>
       </c>
-      <c r="AS5">
+      <c r="AS5" s="0">
         <f>IFERROR(AQ5*U5/T5,0)</f>
         <v/>
       </c>
-      <c r="AT5">
+      <c r="AT5" s="0">
         <f>IF(AND(C5="SEG-03",H5&gt;0),IF(J5&lt;4,0.65,IF(J5&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU5">
+      <c r="AU5" s="0">
         <f>I5*AT5</f>
         <v/>
       </c>
-      <c r="AV5">
+      <c r="AV5" s="0">
         <f>'Lotes_Pipeline_sim2'!AY2+U5</f>
         <v/>
       </c>
-      <c r="AW5">
+      <c r="AW5" s="0">
         <f>MIN(AV5,MAX(0,'Mercados_Pipeline_sim2'!I4))</f>
         <v/>
       </c>
-      <c r="AX5">
+      <c r="AX5" s="0">
         <f>AW5*AU5</f>
         <v/>
       </c>
-      <c r="AY5">
+      <c r="AY5" s="0">
         <f>AV5-AW5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="F6" s="0" t="inlineStr"/>
+      <c r="G6" s="0" t="inlineStr"/>
+      <c r="H6" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E6,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F6,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G6,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D6,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K6">
+      <c r="K6" s="0">
         <f>'Pipeline_sim2'!CG5</f>
         <v/>
       </c>
-      <c r="L6">
+      <c r="L6" s="0">
         <f>'Pipeline_sim2'!CI5</f>
         <v/>
       </c>
-      <c r="M6">
+      <c r="M6" s="0">
         <f>'Pipeline_sim2'!CK5</f>
         <v/>
       </c>
-      <c r="N6">
+      <c r="N6" s="0">
         <f>'Pipeline_sim2'!CM5</f>
         <v/>
       </c>
-      <c r="O6">
+      <c r="O6" s="0">
         <f>'Pipeline_sim2'!CO5</f>
         <v/>
       </c>
-      <c r="P6">
+      <c r="P6" s="0">
         <f>'Pipeline_sim2'!CQ5</f>
         <v/>
       </c>
-      <c r="Q6">
+      <c r="Q6" s="0">
         <f>'Pipeline_sim2'!CS5</f>
         <v/>
       </c>
-      <c r="R6">
+      <c r="R6" s="0">
         <f>'Pipeline_sim2'!CU5</f>
         <v/>
       </c>
-      <c r="S6">
+      <c r="S6" s="0">
         <f>IFERROR(ROUNDDOWN(H6*'Pipeline_sim2'!CE5/'Pipeline_sim2'!I5,0),0)</f>
         <v/>
       </c>
-      <c r="T6">
+      <c r="T6" s="0">
         <f>ROUNDDOWN(MIN(H6,S6,(K6)/0.3,(N6+O6)/1,(P6+Q6+R6)/6),0)</f>
         <v/>
       </c>
-      <c r="U6">
+      <c r="U6" s="0">
         <f>ROUNDDOWN(T6*'Pipeline_sim2'!AU5,0)</f>
         <v/>
       </c>
-      <c r="V6">
+      <c r="V6" s="0">
         <f>MIN(K6,MAX(0,T6*0.3))</f>
         <v/>
       </c>
-      <c r="W6">
+      <c r="W6" s="0">
         <f>K6-V6</f>
         <v/>
       </c>
-      <c r="X6">
+      <c r="X6" s="0">
         <f>IFERROR(V6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="Y6">
+      <c r="Y6" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z6">
+      <c r="Z6" s="0">
         <f>L6-Y6</f>
         <v/>
       </c>
-      <c r="AA6">
+      <c r="AA6" s="0">
         <f>IFERROR(Y6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AB6">
+      <c r="AB6" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC6">
+      <c r="AC6" s="0">
         <f>M6-AB6</f>
         <v/>
       </c>
-      <c r="AD6">
+      <c r="AD6" s="0">
         <f>IFERROR(AB6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AE6">
+      <c r="AE6" s="0">
         <f>MIN(N6,MAX(0,T6*1))</f>
         <v/>
       </c>
-      <c r="AF6">
+      <c r="AF6" s="0">
         <f>N6-AE6</f>
         <v/>
       </c>
-      <c r="AG6">
+      <c r="AG6" s="0">
         <f>IFERROR(AE6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AH6">
+      <c r="AH6" s="0">
         <f>MIN(O6,MAX(0,T6*1-(AE6)))</f>
         <v/>
       </c>
-      <c r="AI6">
+      <c r="AI6" s="0">
         <f>O6-AH6</f>
         <v/>
       </c>
-      <c r="AJ6">
+      <c r="AJ6" s="0">
         <f>IFERROR(AH6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AK6">
+      <c r="AK6" s="0">
         <f>MIN(P6,MAX(0,T6*6))</f>
         <v/>
       </c>
-      <c r="AL6">
+      <c r="AL6" s="0">
         <f>P6-AK6</f>
         <v/>
       </c>
-      <c r="AM6">
+      <c r="AM6" s="0">
         <f>IFERROR(AK6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AN6">
+      <c r="AN6" s="0">
         <f>MIN(Q6,MAX(0,T6*6-(AK6)))</f>
         <v/>
       </c>
-      <c r="AO6">
+      <c r="AO6" s="0">
         <f>Q6-AN6</f>
         <v/>
       </c>
-      <c r="AP6">
+      <c r="AP6" s="0">
         <f>IFERROR(AN6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AQ6">
+      <c r="AQ6" s="0">
         <f>MIN(R6,MAX(0,T6*6-(AK6+AN6)))</f>
         <v/>
       </c>
-      <c r="AR6">
+      <c r="AR6" s="0">
         <f>R6-AQ6</f>
         <v/>
       </c>
-      <c r="AS6">
+      <c r="AS6" s="0">
         <f>IFERROR(AQ6*U6/T6,0)</f>
         <v/>
       </c>
-      <c r="AT6">
+      <c r="AT6" s="0">
         <f>IF(AND(C6="SEG-03",H6&gt;0),IF(J6&lt;4,0.65,IF(J6&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU6">
+      <c r="AU6" s="0">
         <f>I6*AT6</f>
         <v/>
       </c>
-      <c r="AV6">
+      <c r="AV6" s="0">
         <f>'Lotes_Pipeline_sim2'!AY3+U6</f>
         <v/>
       </c>
-      <c r="AW6">
+      <c r="AW6" s="0">
         <f>MIN(AV6,MAX(0,'Mercados_Pipeline_sim2'!I5))</f>
         <v/>
       </c>
-      <c r="AX6">
+      <c r="AX6" s="0">
         <f>AW6*AU6</f>
         <v/>
       </c>
-      <c r="AY6">
+      <c r="AY6" s="0">
         <f>AV6-AW6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
         <is>
           <t>INS-04</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>INS-06</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E7,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F7,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G7,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D7,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K7">
+      <c r="K7" s="0">
         <f>'Lotes_Pipeline_sim2'!W6</f>
         <v/>
       </c>
-      <c r="L7">
+      <c r="L7" s="0">
         <f>'Lotes_Pipeline_sim2'!Z6</f>
         <v/>
       </c>
-      <c r="M7">
+      <c r="M7" s="0">
         <f>'Lotes_Pipeline_sim2'!AC6</f>
         <v/>
       </c>
-      <c r="N7">
+      <c r="N7" s="0">
         <f>'Lotes_Pipeline_sim2'!AF6</f>
         <v/>
       </c>
-      <c r="O7">
+      <c r="O7" s="0">
         <f>'Lotes_Pipeline_sim2'!AI6</f>
         <v/>
       </c>
-      <c r="P7">
+      <c r="P7" s="0">
         <f>'Lotes_Pipeline_sim2'!AL6</f>
         <v/>
       </c>
-      <c r="Q7">
+      <c r="Q7" s="0">
         <f>'Lotes_Pipeline_sim2'!AO6</f>
         <v/>
       </c>
-      <c r="R7">
+      <c r="R7" s="0">
         <f>'Lotes_Pipeline_sim2'!AR6</f>
         <v/>
       </c>
-      <c r="S7">
+      <c r="S7" s="0">
         <f>IFERROR(ROUNDDOWN(H7*'Pipeline_sim2'!CE5/'Pipeline_sim2'!I5,0),0)</f>
         <v/>
       </c>
-      <c r="T7">
+      <c r="T7" s="0">
         <f>ROUNDDOWN(MIN(H7,S7,(K7)/0.3,(N7)/1,(P7)/6),0)</f>
         <v/>
       </c>
-      <c r="U7">
+      <c r="U7" s="0">
         <f>ROUNDDOWN(T7*'Pipeline_sim2'!AU5,0)</f>
         <v/>
       </c>
-      <c r="V7">
+      <c r="V7" s="0">
         <f>MIN(K7,MAX(0,T7*0.3))</f>
         <v/>
       </c>
-      <c r="W7">
+      <c r="W7" s="0">
         <f>K7-V7</f>
         <v/>
       </c>
-      <c r="X7">
+      <c r="X7" s="0">
         <f>IFERROR(V7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="Y7">
+      <c r="Y7" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z7">
+      <c r="Z7" s="0">
         <f>L7-Y7</f>
         <v/>
       </c>
-      <c r="AA7">
+      <c r="AA7" s="0">
         <f>IFERROR(Y7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AB7">
+      <c r="AB7" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC7">
+      <c r="AC7" s="0">
         <f>M7-AB7</f>
         <v/>
       </c>
-      <c r="AD7">
+      <c r="AD7" s="0">
         <f>IFERROR(AB7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AE7">
+      <c r="AE7" s="0">
         <f>MIN(N7,MAX(0,T7*1))</f>
         <v/>
       </c>
-      <c r="AF7">
+      <c r="AF7" s="0">
         <f>N7-AE7</f>
         <v/>
       </c>
-      <c r="AG7">
+      <c r="AG7" s="0">
         <f>IFERROR(AE7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AH7">
+      <c r="AH7" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AI7">
+      <c r="AI7" s="0">
         <f>O7-AH7</f>
         <v/>
       </c>
-      <c r="AJ7">
+      <c r="AJ7" s="0">
         <f>IFERROR(AH7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AK7">
+      <c r="AK7" s="0">
         <f>MIN(P7,MAX(0,T7*6))</f>
         <v/>
       </c>
-      <c r="AL7">
+      <c r="AL7" s="0">
         <f>P7-AK7</f>
         <v/>
       </c>
-      <c r="AM7">
+      <c r="AM7" s="0">
         <f>IFERROR(AK7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AN7">
+      <c r="AN7" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO7">
+      <c r="AO7" s="0">
         <f>Q7-AN7</f>
         <v/>
       </c>
-      <c r="AP7">
+      <c r="AP7" s="0">
         <f>IFERROR(AN7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AQ7">
+      <c r="AQ7" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AR7">
+      <c r="AR7" s="0">
         <f>R7-AQ7</f>
         <v/>
       </c>
-      <c r="AS7">
+      <c r="AS7" s="0">
         <f>IFERROR(AQ7*U7/T7,0)</f>
         <v/>
       </c>
-      <c r="AT7">
+      <c r="AT7" s="0">
         <f>IF(AND(C7="SEG-03",H7&gt;0),IF(J7&lt;4,0.65,IF(J7&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU7">
+      <c r="AU7" s="0">
         <f>I7*AT7</f>
         <v/>
       </c>
-      <c r="AV7">
+      <c r="AV7" s="0">
         <f>'Lotes_Pipeline_sim2'!AY4+U7</f>
         <v/>
       </c>
-      <c r="AW7">
+      <c r="AW7" s="0">
         <f>MIN(AV7,MAX(0,'Mercados_Pipeline_sim2'!I5-('Lotes_Pipeline_sim2'!AW6)))</f>
         <v/>
       </c>
-      <c r="AX7">
+      <c r="AX7" s="0">
         <f>AW7*AU7</f>
         <v/>
       </c>
-      <c r="AY7">
+      <c r="AY7" s="0">
         <f>AV7-AW7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>INF-10</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>INS-03</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="0" t="inlineStr">
         <is>
           <t>INS-05</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>INS-08</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="0" t="n">
         <v>200</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E8,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F8,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G8,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D8,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K8">
+      <c r="K8" s="0">
         <f>'Pipeline_sim2'!CG6</f>
         <v/>
       </c>
-      <c r="L8">
+      <c r="L8" s="0">
         <f>'Pipeline_sim2'!CI6</f>
         <v/>
       </c>
-      <c r="M8">
+      <c r="M8" s="0">
         <f>'Pipeline_sim2'!CK6</f>
         <v/>
       </c>
-      <c r="N8">
+      <c r="N8" s="0">
         <f>'Pipeline_sim2'!CM6</f>
         <v/>
       </c>
-      <c r="O8">
+      <c r="O8" s="0">
         <f>'Pipeline_sim2'!CO6</f>
         <v/>
       </c>
-      <c r="P8">
+      <c r="P8" s="0">
         <f>'Pipeline_sim2'!CQ6</f>
         <v/>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="0">
         <f>'Pipeline_sim2'!CS6</f>
         <v/>
       </c>
-      <c r="R8">
+      <c r="R8" s="0">
         <f>'Pipeline_sim2'!CU6</f>
         <v/>
       </c>
-      <c r="S8">
+      <c r="S8" s="0">
         <f>IFERROR(ROUNDDOWN(H8*'Pipeline_sim2'!CE6/'Pipeline_sim2'!I6,0),0)</f>
         <v/>
       </c>
-      <c r="T8">
+      <c r="T8" s="0">
         <f>ROUNDDOWN(MIN(H8,S8,(M8)/0.7,(O8)/1,(R8)/13),0)</f>
         <v/>
       </c>
-      <c r="U8">
+      <c r="U8" s="0">
         <f>ROUNDDOWN(T8*'Pipeline_sim2'!AU6,0)</f>
         <v/>
       </c>
-      <c r="V8">
+      <c r="V8" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="W8">
+      <c r="W8" s="0">
         <f>K8-V8</f>
         <v/>
       </c>
-      <c r="X8">
+      <c r="X8" s="0">
         <f>IFERROR(V8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="Y8">
+      <c r="Y8" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z8">
+      <c r="Z8" s="0">
         <f>L8-Y8</f>
         <v/>
       </c>
-      <c r="AA8">
+      <c r="AA8" s="0">
         <f>IFERROR(Y8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AB8">
+      <c r="AB8" s="0">
         <f>MIN(M8,MAX(0,T8*0.7-(V8+Y8)))</f>
         <v/>
       </c>
-      <c r="AC8">
+      <c r="AC8" s="0">
         <f>M8-AB8</f>
         <v/>
       </c>
-      <c r="AD8">
+      <c r="AD8" s="0">
         <f>IFERROR(AB8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AE8">
+      <c r="AE8" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AF8">
+      <c r="AF8" s="0">
         <f>N8-AE8</f>
         <v/>
       </c>
-      <c r="AG8">
+      <c r="AG8" s="0">
         <f>IFERROR(AE8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AH8">
+      <c r="AH8" s="0">
         <f>MIN(O8,MAX(0,T8*1-(AE8)))</f>
         <v/>
       </c>
-      <c r="AI8">
+      <c r="AI8" s="0">
         <f>O8-AH8</f>
         <v/>
       </c>
-      <c r="AJ8">
+      <c r="AJ8" s="0">
         <f>IFERROR(AH8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AK8">
+      <c r="AK8" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AL8">
+      <c r="AL8" s="0">
         <f>P8-AK8</f>
         <v/>
       </c>
-      <c r="AM8">
+      <c r="AM8" s="0">
         <f>IFERROR(AK8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AN8">
+      <c r="AN8" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO8">
+      <c r="AO8" s="0">
         <f>Q8-AN8</f>
         <v/>
       </c>
-      <c r="AP8">
+      <c r="AP8" s="0">
         <f>IFERROR(AN8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AQ8">
+      <c r="AQ8" s="0">
         <f>MIN(R8,MAX(0,T8*13-(AK8+AN8)))</f>
         <v/>
       </c>
-      <c r="AR8">
+      <c r="AR8" s="0">
         <f>R8-AQ8</f>
         <v/>
       </c>
-      <c r="AS8">
+      <c r="AS8" s="0">
         <f>IFERROR(AQ8*U8/T8,0)</f>
         <v/>
       </c>
-      <c r="AT8">
+      <c r="AT8" s="0">
         <f>IF(AND(C8="SEG-03",H8&gt;0),IF(J8&lt;4,0.65,IF(J8&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU8">
+      <c r="AU8" s="0">
         <f>I8*AT8</f>
         <v/>
       </c>
-      <c r="AV8">
+      <c r="AV8" s="0">
         <f>'Lotes_Pipeline_sim2'!AY5+U8</f>
         <v/>
       </c>
-      <c r="AW8">
+      <c r="AW8" s="0">
         <f>MIN(AV8,MAX(0,'Mercados_Pipeline_sim2'!I6))</f>
         <v/>
       </c>
-      <c r="AX8">
+      <c r="AX8" s="0">
         <f>AW8*AU8</f>
         <v/>
       </c>
-      <c r="AY8">
+      <c r="AY8" s="0">
         <f>AV8-AW8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="F9" s="0" t="inlineStr"/>
+      <c r="G9" s="0" t="inlineStr"/>
+      <c r="H9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E9,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F9,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G9,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D9,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K9">
+      <c r="K9" s="0">
         <f>'Pipeline_sim2'!CG7</f>
         <v/>
       </c>
-      <c r="L9">
+      <c r="L9" s="0">
         <f>'Pipeline_sim2'!CI7</f>
         <v/>
       </c>
-      <c r="M9">
+      <c r="M9" s="0">
         <f>'Pipeline_sim2'!CK7</f>
         <v/>
       </c>
-      <c r="N9">
+      <c r="N9" s="0">
         <f>'Pipeline_sim2'!CM7</f>
         <v/>
       </c>
-      <c r="O9">
+      <c r="O9" s="0">
         <f>'Pipeline_sim2'!CO7</f>
         <v/>
       </c>
-      <c r="P9">
+      <c r="P9" s="0">
         <f>'Pipeline_sim2'!CQ7</f>
         <v/>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="0">
         <f>'Pipeline_sim2'!CS7</f>
         <v/>
       </c>
-      <c r="R9">
+      <c r="R9" s="0">
         <f>'Pipeline_sim2'!CU7</f>
         <v/>
       </c>
-      <c r="S9">
+      <c r="S9" s="0">
         <f>IFERROR(ROUNDDOWN(H9*'Pipeline_sim2'!CE7/'Pipeline_sim2'!I7,0),0)</f>
         <v/>
       </c>
-      <c r="T9">
+      <c r="T9" s="0">
         <f>ROUNDDOWN(MIN(H9,S9,(K9)/0.3,(N9+O9)/1,(P9+Q9+R9)/6),0)</f>
         <v/>
       </c>
-      <c r="U9">
+      <c r="U9" s="0">
         <f>ROUNDDOWN(T9*'Pipeline_sim2'!AU7,0)</f>
         <v/>
       </c>
-      <c r="V9">
+      <c r="V9" s="0">
         <f>MIN(K9,MAX(0,T9*0.3))</f>
         <v/>
       </c>
-      <c r="W9">
+      <c r="W9" s="0">
         <f>K9-V9</f>
         <v/>
       </c>
-      <c r="X9">
+      <c r="X9" s="0">
         <f>IFERROR(V9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="Y9">
+      <c r="Y9" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z9">
+      <c r="Z9" s="0">
         <f>L9-Y9</f>
         <v/>
       </c>
-      <c r="AA9">
+      <c r="AA9" s="0">
         <f>IFERROR(Y9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AB9">
+      <c r="AB9" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC9">
+      <c r="AC9" s="0">
         <f>M9-AB9</f>
         <v/>
       </c>
-      <c r="AD9">
+      <c r="AD9" s="0">
         <f>IFERROR(AB9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AE9">
+      <c r="AE9" s="0">
         <f>MIN(N9,MAX(0,T9*1))</f>
         <v/>
       </c>
-      <c r="AF9">
+      <c r="AF9" s="0">
         <f>N9-AE9</f>
         <v/>
       </c>
-      <c r="AG9">
+      <c r="AG9" s="0">
         <f>IFERROR(AE9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AH9">
+      <c r="AH9" s="0">
         <f>MIN(O9,MAX(0,T9*1-(AE9)))</f>
         <v/>
       </c>
-      <c r="AI9">
+      <c r="AI9" s="0">
         <f>O9-AH9</f>
         <v/>
       </c>
-      <c r="AJ9">
+      <c r="AJ9" s="0">
         <f>IFERROR(AH9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AK9">
+      <c r="AK9" s="0">
         <f>MIN(P9,MAX(0,T9*6))</f>
         <v/>
       </c>
-      <c r="AL9">
+      <c r="AL9" s="0">
         <f>P9-AK9</f>
         <v/>
       </c>
-      <c r="AM9">
+      <c r="AM9" s="0">
         <f>IFERROR(AK9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AN9">
+      <c r="AN9" s="0">
         <f>MIN(Q9,MAX(0,T9*6-(AK9)))</f>
         <v/>
       </c>
-      <c r="AO9">
+      <c r="AO9" s="0">
         <f>Q9-AN9</f>
         <v/>
       </c>
-      <c r="AP9">
+      <c r="AP9" s="0">
         <f>IFERROR(AN9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AQ9">
+      <c r="AQ9" s="0">
         <f>MIN(R9,MAX(0,T9*6-(AK9+AN9)))</f>
         <v/>
       </c>
-      <c r="AR9">
+      <c r="AR9" s="0">
         <f>R9-AQ9</f>
         <v/>
       </c>
-      <c r="AS9">
+      <c r="AS9" s="0">
         <f>IFERROR(AQ9*U9/T9,0)</f>
         <v/>
       </c>
-      <c r="AT9">
+      <c r="AT9" s="0">
         <f>IF(AND(C9="SEG-03",H9&gt;0),IF(J9&lt;4,0.65,IF(J9&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU9">
+      <c r="AU9" s="0">
         <f>'Lotes_Pipeline_sim2'!AU6</f>
         <v/>
       </c>
-      <c r="AV9">
+      <c r="AV9" s="0">
         <f>'Lotes_Pipeline_sim2'!AY6+U9</f>
         <v/>
       </c>
-      <c r="AW9">
+      <c r="AW9" s="0">
         <f>MIN(AV9,MAX(0,'Mercados_Pipeline_sim2'!I8))</f>
         <v/>
       </c>
-      <c r="AX9">
+      <c r="AX9" s="0">
         <f>AW9*AU9</f>
         <v/>
       </c>
-      <c r="AY9">
+      <c r="AY9" s="0">
         <f>AV9-AW9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>INF-08</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>INS-01</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="0" t="inlineStr">
         <is>
           <t>INS-04</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="0" t="inlineStr">
         <is>
           <t>INS-06</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="H10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0" t="n">
         <v>250</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E10,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F10,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G10,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D10,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K10">
+      <c r="K10" s="0">
         <f>'Lotes_Pipeline_sim2'!W9</f>
         <v/>
       </c>
-      <c r="L10">
+      <c r="L10" s="0">
         <f>'Lotes_Pipeline_sim2'!Z9</f>
         <v/>
       </c>
-      <c r="M10">
+      <c r="M10" s="0">
         <f>'Lotes_Pipeline_sim2'!AC9</f>
         <v/>
       </c>
-      <c r="N10">
+      <c r="N10" s="0">
         <f>'Lotes_Pipeline_sim2'!AF9</f>
         <v/>
       </c>
-      <c r="O10">
+      <c r="O10" s="0">
         <f>'Lotes_Pipeline_sim2'!AI9</f>
         <v/>
       </c>
-      <c r="P10">
+      <c r="P10" s="0">
         <f>'Lotes_Pipeline_sim2'!AL9</f>
         <v/>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="0">
         <f>'Lotes_Pipeline_sim2'!AO9</f>
         <v/>
       </c>
-      <c r="R10">
+      <c r="R10" s="0">
         <f>'Lotes_Pipeline_sim2'!AR9</f>
         <v/>
       </c>
-      <c r="S10">
+      <c r="S10" s="0">
         <f>IFERROR(ROUNDDOWN(H10*'Pipeline_sim2'!CE7/'Pipeline_sim2'!I7,0),0)</f>
         <v/>
       </c>
-      <c r="T10">
+      <c r="T10" s="0">
         <f>ROUNDDOWN(MIN(H10,S10,(K10)/0.3,(N10)/1,(P10)/6),0)</f>
         <v/>
       </c>
-      <c r="U10">
+      <c r="U10" s="0">
         <f>ROUNDDOWN(T10*'Pipeline_sim2'!AU7,0)</f>
         <v/>
       </c>
-      <c r="V10">
+      <c r="V10" s="0">
         <f>MIN(K10,MAX(0,T10*0.3))</f>
         <v/>
       </c>
-      <c r="W10">
+      <c r="W10" s="0">
         <f>K10-V10</f>
         <v/>
       </c>
-      <c r="X10">
+      <c r="X10" s="0">
         <f>IFERROR(V10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="Y10">
+      <c r="Y10" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z10">
+      <c r="Z10" s="0">
         <f>L10-Y10</f>
         <v/>
       </c>
-      <c r="AA10">
+      <c r="AA10" s="0">
         <f>IFERROR(Y10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AB10">
+      <c r="AB10" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AC10">
+      <c r="AC10" s="0">
         <f>M10-AB10</f>
         <v/>
       </c>
-      <c r="AD10">
+      <c r="AD10" s="0">
         <f>IFERROR(AB10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AE10">
+      <c r="AE10" s="0">
         <f>MIN(N10,MAX(0,T10*1))</f>
         <v/>
       </c>
-      <c r="AF10">
+      <c r="AF10" s="0">
         <f>N10-AE10</f>
         <v/>
       </c>
-      <c r="AG10">
+      <c r="AG10" s="0">
         <f>IFERROR(AE10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AH10">
+      <c r="AH10" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AI10">
+      <c r="AI10" s="0">
         <f>O10-AH10</f>
         <v/>
       </c>
-      <c r="AJ10">
+      <c r="AJ10" s="0">
         <f>IFERROR(AH10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AK10">
+      <c r="AK10" s="0">
         <f>MIN(P10,MAX(0,T10*6))</f>
         <v/>
       </c>
-      <c r="AL10">
+      <c r="AL10" s="0">
         <f>P10-AK10</f>
         <v/>
       </c>
-      <c r="AM10">
+      <c r="AM10" s="0">
         <f>IFERROR(AK10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AN10">
+      <c r="AN10" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO10">
+      <c r="AO10" s="0">
         <f>Q10-AN10</f>
         <v/>
       </c>
-      <c r="AP10">
+      <c r="AP10" s="0">
         <f>IFERROR(AN10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AQ10">
+      <c r="AQ10" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AR10">
+      <c r="AR10" s="0">
         <f>R10-AQ10</f>
         <v/>
       </c>
-      <c r="AS10">
+      <c r="AS10" s="0">
         <f>IFERROR(AQ10*U10/T10,0)</f>
         <v/>
       </c>
-      <c r="AT10">
+      <c r="AT10" s="0">
         <f>IF(AND(C10="SEG-03",H10&gt;0),IF(J10&lt;4,0.65,IF(J10&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU10">
+      <c r="AU10" s="0">
         <f>'Lotes_Pipeline_sim2'!AU7</f>
         <v/>
       </c>
-      <c r="AV10">
+      <c r="AV10" s="0">
         <f>'Lotes_Pipeline_sim2'!AY7+U10</f>
         <v/>
       </c>
-      <c r="AW10">
+      <c r="AW10" s="0">
         <f>MIN(AV10,MAX(0,'Mercados_Pipeline_sim2'!I8-('Lotes_Pipeline_sim2'!AW9)))</f>
         <v/>
       </c>
-      <c r="AX10">
+      <c r="AX10" s="0">
         <f>AW10*AU10</f>
         <v/>
       </c>
-      <c r="AY10">
+      <c r="AY10" s="0">
         <f>AV10-AW10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>SEG-02</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>INF-09</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>INS-03</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="0" t="inlineStr">
         <is>
           <t>INS-05</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="0" t="inlineStr">
         <is>
           <t>INS-08</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="0">
         <f>IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(E11,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(F11,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(G11,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)+IFERROR(INDEX('Catalogo_Numerico_sim2'!$H$2:$H$69,MATCH(D11,'Catalogo_Numerico_sim2'!$A$2:$A$69,0)),0)</f>
         <v/>
       </c>
-      <c r="K11">
+      <c r="K11" s="0">
         <f>'Lotes_Pipeline_sim2'!W10</f>
         <v/>
       </c>
-      <c r="L11">
+      <c r="L11" s="0">
         <f>'Lotes_Pipeline_sim2'!Z10</f>
         <v/>
       </c>
-      <c r="M11">
+      <c r="M11" s="0">
         <f>'Lotes_Pipeline_sim2'!AC10</f>
         <v/>
       </c>
-      <c r="N11">
+      <c r="N11" s="0">
         <f>'Lotes_Pipeline_sim2'!AF10</f>
         <v/>
       </c>
-      <c r="O11">
+      <c r="O11" s="0">
         <f>'Lotes_Pipeline_sim2'!AI10</f>
         <v/>
       </c>
-      <c r="P11">
+      <c r="P11" s="0">
         <f>'Lotes_Pipeline_sim2'!AL10</f>
         <v/>
       </c>
-      <c r="Q11">
+      <c r="Q11" s="0">
         <f>'Lotes_Pipeline_sim2'!AO10</f>
         <v/>
       </c>
-      <c r="R11">
+      <c r="R11" s="0">
         <f>'Lotes_Pipeline_sim2'!AR10</f>
         <v/>
       </c>
-      <c r="S11">
+      <c r="S11" s="0">
         <f>IFERROR(ROUNDDOWN(H11*'Pipeline_sim2'!CE7/'Pipeline_sim2'!I7,0),0)</f>
         <v/>
       </c>
-      <c r="T11">
+      <c r="T11" s="0">
         <f>ROUNDDOWN(MIN(H11,S11,(M11)/0.4,(O11)/1,(R11)/7),0)</f>
         <v/>
       </c>
-      <c r="U11">
+      <c r="U11" s="0">
         <f>ROUNDDOWN(T11*'Pipeline_sim2'!AU7,0)</f>
         <v/>
       </c>
-      <c r="V11">
+      <c r="V11" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="W11">
+      <c r="W11" s="0">
         <f>K11-V11</f>
         <v/>
       </c>
-      <c r="X11">
+      <c r="X11" s="0">
         <f>IFERROR(V11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="Y11">
+      <c r="Y11" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="Z11">
+      <c r="Z11" s="0">
         <f>L11-Y11</f>
         <v/>
       </c>
-      <c r="AA11">
+      <c r="AA11" s="0">
         <f>IFERROR(Y11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AB11">
+      <c r="AB11" s="0">
         <f>MIN(M11,MAX(0,T11*0.4-(V11+Y11)))</f>
         <v/>
       </c>
-      <c r="AC11">
+      <c r="AC11" s="0">
         <f>M11-AB11</f>
         <v/>
       </c>
-      <c r="AD11">
+      <c r="AD11" s="0">
         <f>IFERROR(AB11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AE11">
+      <c r="AE11" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AF11">
+      <c r="AF11" s="0">
         <f>N11-AE11</f>
         <v/>
       </c>
-      <c r="AG11">
+      <c r="AG11" s="0">
         <f>IFERROR(AE11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AH11">
+      <c r="AH11" s="0">
         <f>MIN(O11,MAX(0,T11*1-(AE11)))</f>
         <v/>
       </c>
-      <c r="AI11">
+      <c r="AI11" s="0">
         <f>O11-AH11</f>
         <v/>
       </c>
-      <c r="AJ11">
+      <c r="AJ11" s="0">
         <f>IFERROR(AH11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AK11">
+      <c r="AK11" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AL11">
+      <c r="AL11" s="0">
         <f>P11-AK11</f>
         <v/>
       </c>
-      <c r="AM11">
+      <c r="AM11" s="0">
         <f>IFERROR(AK11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AN11">
+      <c r="AN11" s="0">
         <f>0</f>
         <v/>
       </c>
-      <c r="AO11">
+      <c r="AO11" s="0">
         <f>Q11-AN11</f>
         <v/>
       </c>
-      <c r="AP11">
+      <c r="AP11" s="0">
         <f>IFERROR(AN11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AQ11">
+      <c r="AQ11" s="0">
         <f>MIN(R11,MAX(0,T11*7-(AK11+AN11)))</f>
         <v/>
       </c>
-      <c r="AR11">
+      <c r="AR11" s="0">
         <f>R11-AQ11</f>
         <v/>
       </c>
-      <c r="AS11">
+      <c r="AS11" s="0">
         <f>IFERROR(AQ11*U11/T11,0)</f>
         <v/>
       </c>
-      <c r="AT11">
+      <c r="AT11" s="0">
         <f>IF(AND(C11="SEG-03",H11&gt;0),IF(J11&lt;4,0.65,IF(J11&gt;=7,1.4,1)),1)</f>
         <v/>
       </c>
-      <c r="AU11">
+      <c r="AU11" s="0">
         <f>I11*AT11</f>
         <v/>
       </c>
-      <c r="AV11">
+      <c r="AV11" s="0">
         <f>0+U11</f>
         <v/>
       </c>
-      <c r="AW11">
+      <c r="AW11" s="0">
         <f>MIN(AV11,MAX(0,'Mercados_Pipeline_sim2'!I7))</f>
         <v/>
       </c>
-      <c r="AX11">
+      <c r="AX11" s="0">
         <f>AW11*AU11</f>
         <v/>
       </c>
-      <c r="AY11">
+      <c r="AY11" s="0">
         <f>AV11-AW11</f>
         <v/>
       </c>
@@ -14784,493 +16170,493 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>ciclo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>empresa</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>segmento</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
         <is>
           <t>precio</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="0" t="inlineStr">
         <is>
           <t>reputacion</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="0" t="inlineStr">
         <is>
           <t>calidad</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="0" t="inlineStr">
         <is>
           <t>demandaAjustada</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="0" t="inlineStr">
         <is>
           <t>asignado</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="0" t="inlineStr">
         <is>
           <t>puntajePrecio</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>puntajeTotal</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="0" t="inlineStr">
         <is>
           <t>reputacionEscalada</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="0" t="inlineStr">
         <is>
           <t>porcentaje</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>1|SEG-03</t>
         </is>
       </c>
-      <c r="E2">
+      <c r="E2" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F2">
+      <c r="F2" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I2*'Lotes_Pipeline_sim2'!H2)/('Lotes_Pipeline_sim2'!H2),0)</f>
         <v/>
       </c>
-      <c r="G2">
+      <c r="G2" s="0">
         <f>'Pipeline_sim2'!DY2</f>
         <v/>
       </c>
-      <c r="H2">
+      <c r="H2" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI2*10),0)</f>
         <v/>
       </c>
-      <c r="I2">
+      <c r="I2" s="0">
         <f>MAX(0,ROUNDDOWN(J2*'Pipeline_sim2'!AN2*1.12,0))</f>
         <v/>
       </c>
-      <c r="J2">
+      <c r="J2" s="0">
         <f>IFERROR(ROUND(L2/SUMIF($D$2:$D$8,D2,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K2">
+      <c r="K2" s="0">
         <f>100-ABS(F2-250)/250*100</f>
         <v/>
       </c>
-      <c r="L2">
+      <c r="L2" s="0">
         <f>IF(E2,0.1*K2+0.5*G2*10+0.4*H2,0)</f>
         <v/>
       </c>
-      <c r="M2">
+      <c r="M2" s="0">
         <f>G2*10</f>
         <v/>
       </c>
-      <c r="N2">
+      <c r="N2" s="0">
         <f>IFERROR(L2/SUMIF($D$2:$D$8,D2,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>1|SEG-03</t>
         </is>
       </c>
-      <c r="E3">
+      <c r="E3" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F3">
+      <c r="F3" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I3*'Lotes_Pipeline_sim2'!H3+'Lotes_Pipeline_sim2'!I4*'Lotes_Pipeline_sim2'!H4)/('Lotes_Pipeline_sim2'!H3+'Lotes_Pipeline_sim2'!H4),0)</f>
         <v/>
       </c>
-      <c r="G3">
+      <c r="G3" s="0">
         <f>'Pipeline_sim2'!DY3</f>
         <v/>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI3*10),0)</f>
         <v/>
       </c>
-      <c r="I3">
+      <c r="I3" s="0">
         <f>MAX(0,ROUNDDOWN(J3*'Pipeline_sim2'!AN3*1,0))</f>
         <v/>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <f>IFERROR(ROUND(L3/SUMIF($D$2:$D$8,D3,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K3">
+      <c r="K3" s="0">
         <f>100-ABS(F3-250)/250*100</f>
         <v/>
       </c>
-      <c r="L3">
+      <c r="L3" s="0">
         <f>IF(E3,0.1*K3+0.5*G3*10+0.4*H3,0)</f>
         <v/>
       </c>
-      <c r="M3">
+      <c r="M3" s="0">
         <f>G3*10</f>
         <v/>
       </c>
-      <c r="N3">
+      <c r="N3" s="0">
         <f>IFERROR(L3/SUMIF($D$2:$D$8,D3,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>2|SEG-03</t>
         </is>
       </c>
-      <c r="E4">
+      <c r="E4" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F4">
+      <c r="F4" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I5*'Lotes_Pipeline_sim2'!H5)/('Lotes_Pipeline_sim2'!H5),0)</f>
         <v/>
       </c>
-      <c r="G4">
+      <c r="G4" s="0">
         <f>'Pipeline_sim2'!DY4</f>
         <v/>
       </c>
-      <c r="H4">
+      <c r="H4" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI4*10),0)</f>
         <v/>
       </c>
-      <c r="I4">
+      <c r="I4" s="0">
         <f>MAX(0,ROUNDDOWN(J4*'Pipeline_sim2'!AN4*1.12,0))</f>
         <v/>
       </c>
-      <c r="J4">
+      <c r="J4" s="0">
         <f>IFERROR(ROUND(L4/SUMIF($D$2:$D$8,D4,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K4">
+      <c r="K4" s="0">
         <f>100-ABS(F4-250)/250*100</f>
         <v/>
       </c>
-      <c r="L4">
+      <c r="L4" s="0">
         <f>IF(E4,0.1*K4+0.5*G4*10+0.4*H4,0)</f>
         <v/>
       </c>
-      <c r="M4">
+      <c r="M4" s="0">
         <f>G4*10</f>
         <v/>
       </c>
-      <c r="N4">
+      <c r="N4" s="0">
         <f>IFERROR(L4/SUMIF($D$2:$D$8,D4,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>2|SEG-03</t>
         </is>
       </c>
-      <c r="E5">
+      <c r="E5" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F5">
+      <c r="F5" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I6*'Lotes_Pipeline_sim2'!H6+'Lotes_Pipeline_sim2'!I7*'Lotes_Pipeline_sim2'!H7)/('Lotes_Pipeline_sim2'!H6+'Lotes_Pipeline_sim2'!H7),0)</f>
         <v/>
       </c>
-      <c r="G5">
+      <c r="G5" s="0">
         <f>'Pipeline_sim2'!DY5</f>
         <v/>
       </c>
-      <c r="H5">
+      <c r="H5" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI5*10),0)</f>
         <v/>
       </c>
-      <c r="I5">
+      <c r="I5" s="0">
         <f>MAX(0,ROUNDDOWN(J5*'Pipeline_sim2'!AN5*1,0))</f>
         <v/>
       </c>
-      <c r="J5">
+      <c r="J5" s="0">
         <f>IFERROR(ROUND(L5/SUMIF($D$2:$D$8,D5,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K5">
+      <c r="K5" s="0">
         <f>100-ABS(F5-250)/250*100</f>
         <v/>
       </c>
-      <c r="L5">
+      <c r="L5" s="0">
         <f>IF(E5,0.1*K5+0.5*G5*10+0.4*H5,0)</f>
         <v/>
       </c>
-      <c r="M5">
+      <c r="M5" s="0">
         <f>G5*10</f>
         <v/>
       </c>
-      <c r="N5">
+      <c r="N5" s="0">
         <f>IFERROR(L5/SUMIF($D$2:$D$8,D5,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>3|SEG-03</t>
         </is>
       </c>
-      <c r="E6">
+      <c r="E6" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I8*'Lotes_Pipeline_sim2'!H8)/('Lotes_Pipeline_sim2'!H8),0)</f>
         <v/>
       </c>
-      <c r="G6">
+      <c r="G6" s="0">
         <f>'Pipeline_sim2'!DY6</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="H6" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI6*10),0)</f>
         <v/>
       </c>
-      <c r="I6">
+      <c r="I6" s="0">
         <f>MAX(0,ROUNDDOWN(J6*'Pipeline_sim2'!AN6*1.12,0))</f>
         <v/>
       </c>
-      <c r="J6">
+      <c r="J6" s="0">
         <f>IFERROR(ROUND(L6/SUMIF($D$2:$D$8,D6,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K6">
+      <c r="K6" s="0">
         <f>100-ABS(F6-250)/250*100</f>
         <v/>
       </c>
-      <c r="L6">
+      <c r="L6" s="0">
         <f>IF(E6,0.1*K6+0.5*G6*10+0.4*H6,0)</f>
         <v/>
       </c>
-      <c r="M6">
+      <c r="M6" s="0">
         <f>G6*10</f>
         <v/>
       </c>
-      <c r="N6">
+      <c r="N6" s="0">
         <f>IFERROR(L6/SUMIF($D$2:$D$8,D6,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>SEG-02</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>3|SEG-02</t>
         </is>
       </c>
-      <c r="E7">
+      <c r="E7" s="0">
         <f>TRUE()</f>
         <v/>
       </c>
-      <c r="F7">
+      <c r="F7" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I11*'Lotes_Pipeline_sim2'!H11)/('Lotes_Pipeline_sim2'!H11),0)</f>
         <v/>
       </c>
-      <c r="G7">
+      <c r="G7" s="0">
         <f>'Pipeline_sim2'!DY7</f>
         <v/>
       </c>
-      <c r="H7">
+      <c r="H7" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI7*10),0)</f>
         <v/>
       </c>
-      <c r="I7">
+      <c r="I7" s="0">
         <f>MAX(0,ROUNDDOWN(J7*'Pipeline_sim2'!AN7*1,0))</f>
         <v/>
       </c>
-      <c r="J7">
+      <c r="J7" s="0">
         <f>IFERROR(ROUND(L7/SUMIF($D$2:$D$8,D7,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K7">
+      <c r="K7" s="0">
         <f>100-ABS(F7-100)/100*100</f>
         <v/>
       </c>
-      <c r="L7">
+      <c r="L7" s="0">
         <f>IF(E7,0.4*K7+0.35*G7*10+0.25*H7,0)</f>
         <v/>
       </c>
-      <c r="M7">
+      <c r="M7" s="0">
         <f>G7*10</f>
         <v/>
       </c>
-      <c r="N7">
+      <c r="N7" s="0">
         <f>IFERROR(L7/SUMIF($D$2:$D$8,D7,$L$2:$L$8),0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>SEG-03</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>3|SEG-03</t>
         </is>
       </c>
-      <c r="E8">
+      <c r="E8" s="0">
         <f>('Lotes_Pipeline_sim2'!AV9+'Lotes_Pipeline_sim2'!AV10)&gt;0</f>
         <v/>
       </c>
-      <c r="F8">
+      <c r="F8" s="0">
         <f>IFERROR(('Lotes_Pipeline_sim2'!I9*'Lotes_Pipeline_sim2'!AV9+'Lotes_Pipeline_sim2'!I10*'Lotes_Pipeline_sim2'!AV10)/('Lotes_Pipeline_sim2'!AV9+'Lotes_Pipeline_sim2'!AV10),0)</f>
         <v/>
       </c>
-      <c r="G8">
+      <c r="G8" s="0">
         <f>'Pipeline_sim2'!DY7</f>
         <v/>
       </c>
-      <c r="H8">
+      <c r="H8" s="0">
         <f>ROUND(MIN(100,'Pipeline_sim2'!AI7*10),0)</f>
         <v/>
       </c>
-      <c r="I8">
+      <c r="I8" s="0">
         <f>MAX(0,ROUNDDOWN(J8*'Pipeline_sim2'!AN7*1,0))</f>
         <v/>
       </c>
-      <c r="J8">
+      <c r="J8" s="0">
         <f>IFERROR(ROUND(L8/SUMIF($D$2:$D$8,D8,$L$2:$L$8)*10*1,0),0)</f>
         <v/>
       </c>
-      <c r="K8">
+      <c r="K8" s="0">
         <f>100-ABS(F8-250)/250*100</f>
         <v/>
       </c>
-      <c r="L8">
+      <c r="L8" s="0">
         <f>IF(E8,0.1*K8+0.5*G8*10+0.4*H8,0)</f>
         <v/>
       </c>
-      <c r="M8">
+      <c r="M8" s="0">
         <f>G8*10</f>
         <v/>
       </c>
-      <c r="N8">
+      <c r="N8" s="0">
         <f>IFERROR(L8/SUMIF($D$2:$D$8,D8,$L$2:$L$8),0)</f>
         <v/>
       </c>

</xml_diff>